<commit_message>
Ajout CADENCIER.xlsx – 69 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8877" uniqueCount="4503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9025" uniqueCount="4581">
   <si>
     <t>Code barre</t>
   </si>
@@ -13520,6 +13520,240 @@
   </si>
   <si>
     <t>FARINE MULTIUSAGE FIONA 1KG</t>
+  </si>
+  <si>
+    <t>TAILLE CRAYON COUL ASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHANDARANA </t>
+  </si>
+  <si>
+    <t>COLLE BLANCHE 120ML</t>
+  </si>
+  <si>
+    <t>COLLE BATON 20G</t>
+  </si>
+  <si>
+    <t>PAINTING PALETTE 14 COMP 190MM</t>
+  </si>
+  <si>
+    <t>TROUSSE 210X85X45MM BLEU FONCE</t>
+  </si>
+  <si>
+    <t>TROUSSE 210X85X45MM ROSE</t>
+  </si>
+  <si>
+    <t>TROUSSE  COUL ASS 19X5X5CM</t>
+  </si>
+  <si>
+    <t>GOUACHE 18 COUL 12ML</t>
+  </si>
+  <si>
+    <t>CRAYON DE 12 COUL COLOR RUN</t>
+  </si>
+  <si>
+    <t>PEINTURE A L'EAU 12COUL</t>
+  </si>
+  <si>
+    <t>FEUTRE 12 COULEUR</t>
+  </si>
+  <si>
+    <t>PAPIER PHOTOCOPIE A4 GLOBAL</t>
+  </si>
+  <si>
+    <t>BLANCO ROLLER 5X12MM ASS</t>
+  </si>
+  <si>
+    <t>REGLE 4PCS COMPLET 30CM BLUE</t>
+  </si>
+  <si>
+    <t>REGLE FLEXIBLE 30CM</t>
+  </si>
+  <si>
+    <t>CITRONNELLE SECHEE 20G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIDJINN </t>
+  </si>
+  <si>
+    <t>CUMIN MOULU 50G</t>
+  </si>
+  <si>
+    <t>CURRY DOUX 15 EPICES</t>
+  </si>
+  <si>
+    <t>PIMENT MOULU</t>
+  </si>
+  <si>
+    <t>MARGARINE PASTEURISEE EN BRQT 250G</t>
+  </si>
+  <si>
+    <t>BISCUITS FINGO 10 ENROBES DE CHOCOLAT</t>
+  </si>
+  <si>
+    <t>BISCUITS FINGO 5 ENROBES DE CHOCOLAT</t>
+  </si>
+  <si>
+    <t>BISCUIT BIS'NICE 9 54G</t>
+  </si>
+  <si>
+    <t>NOUILLE PRESTO SUPREME 92G</t>
+  </si>
+  <si>
+    <t>YAOURT A BOIRE 150ML</t>
+  </si>
+  <si>
+    <t>YAO POP FRAISE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JB </t>
+  </si>
+  <si>
+    <t>YAO POP FRAMBOISE</t>
+  </si>
+  <si>
+    <t>FANTA LIMONADE 1,5L</t>
+  </si>
+  <si>
+    <t>FANTA LIMONADE 350 ML</t>
+  </si>
+  <si>
+    <t>NOUILLE TRADITIONELLE VOKY B 200G POULET PIQUANT</t>
+  </si>
+  <si>
+    <t>NOUILLE TRADITIONELLE VOKY B 200G POULET SPICY</t>
+  </si>
+  <si>
+    <t>NOUILLE TRADITIONELLE VOKY B 200G SAVEUR BOEUF</t>
+  </si>
+  <si>
+    <t>NOUILLE TRADITIONELLE VOKY B 200 GRAMMES TOM YUM</t>
+  </si>
+  <si>
+    <t>CARRY MOULU DOYPACK 30G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAF </t>
+  </si>
+  <si>
+    <t>POIVRE MOULU DOYPACK 30G</t>
+  </si>
+  <si>
+    <t>SAVON HERBAL ACTIVE HYGIENE 100G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AZIMA </t>
+  </si>
+  <si>
+    <t>SAVON CARE ACTIVE HYGIENNE 100G</t>
+  </si>
+  <si>
+    <t>SAVON ACTIVE ACTIVE HYGIENNE 100G</t>
+  </si>
+  <si>
+    <t>SAVON FRESH ACTIVE HYGIENNE 100G</t>
+  </si>
+  <si>
+    <t>MAQ LESSIVE EN POUDRE 500G</t>
+  </si>
+  <si>
+    <t>MAQ LESSIVE EN POUDRE 100G</t>
+  </si>
+  <si>
+    <t>MAQ DETERGENT EN POUDRE 30G</t>
+  </si>
+  <si>
+    <t>SEVRI NATURE SACHET DE 300G</t>
+  </si>
+  <si>
+    <t>FY DELICIEUX</t>
+  </si>
+  <si>
+    <t>SEVRI MELANGE SACHET DE 300G</t>
+  </si>
+  <si>
+    <t>SEVRI PIMENTE SACHET DE 300G</t>
+  </si>
+  <si>
+    <t>SEVRI NATURE BARQUETTE DE 300G</t>
+  </si>
+  <si>
+    <t>SEVRI MELANGE BARQUETTE DE 300G</t>
+  </si>
+  <si>
+    <t>SEVRI PIMENTE BARQUETTE DE 300G</t>
+  </si>
+  <si>
+    <t>DOYPACK BAOBAB 50G</t>
+  </si>
+  <si>
+    <t>GREENCAY</t>
+  </si>
+  <si>
+    <t>DOYPACK PIMENT BEC D'OISEAU 50G</t>
+  </si>
+  <si>
+    <t>DOYPACK CANNELLES EN BATONS 50G</t>
+  </si>
+  <si>
+    <t>DOYPACK CANELLES EN POUDRE 50G</t>
+  </si>
+  <si>
+    <t>DOYPACK CLOU DE GIROFLE 50G</t>
+  </si>
+  <si>
+    <t>DOYPACK COMBAVA 50G</t>
+  </si>
+  <si>
+    <t>DOYPACK PAPRIKA  50G</t>
+  </si>
+  <si>
+    <t>MIEL EUCALYPTUS BOCAL 200ML</t>
+  </si>
+  <si>
+    <t>MIEL MULTIFLORALES BOCAL 200ML</t>
+  </si>
+  <si>
+    <t>CAPRICE CITRON PET 50 CL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STAR </t>
+  </si>
+  <si>
+    <t>CAPRICE CITRON PET 150 CL</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER DEDESSIN 16P PF</t>
+  </si>
+  <si>
+    <t>PAPETERIE ET BUREAUTIQUE MODERNE</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER ECRITURE 32P PF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER 96P PF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER 192P PF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER 96P GF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER 192P GF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER POLYPRO 96P PF</t>
+  </si>
+  <si>
+    <t>TROPHEE CAHIER POLYPRO 192P PF</t>
+  </si>
+  <si>
+    <t>TROPHEE STYLO  GLOSSY</t>
+  </si>
+  <si>
+    <t>TROPHEE STYLO POLO</t>
   </si>
 </sst>
 </file>
@@ -13896,7 +14130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2258"/>
+  <dimension ref="A1:E2327"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -52285,6 +52519,1179 @@
         <v>30</v>
       </c>
     </row>
+    <row r="2259" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2259">
+        <v>6921734905604</v>
+      </c>
+      <c r="B2259">
+        <v>74093662</v>
+      </c>
+      <c r="C2259" t="s">
+        <v>4503</v>
+      </c>
+      <c r="D2259">
+        <v>1</v>
+      </c>
+      <c r="E2259" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2260" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2260">
+        <v>6935205394477</v>
+      </c>
+      <c r="B2260">
+        <v>74093676</v>
+      </c>
+      <c r="C2260" t="s">
+        <v>4505</v>
+      </c>
+      <c r="D2260">
+        <v>1</v>
+      </c>
+      <c r="E2260" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2261">
+        <v>6935205388735</v>
+      </c>
+      <c r="B2261">
+        <v>74093677</v>
+      </c>
+      <c r="C2261" t="s">
+        <v>4506</v>
+      </c>
+      <c r="D2261">
+        <v>1</v>
+      </c>
+      <c r="E2261" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2262" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2262">
+        <v>6935205362643</v>
+      </c>
+      <c r="B2262">
+        <v>74093678</v>
+      </c>
+      <c r="C2262" t="s">
+        <v>4507</v>
+      </c>
+      <c r="D2262">
+        <v>1</v>
+      </c>
+      <c r="E2262" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2263" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2263">
+        <v>6975165332423</v>
+      </c>
+      <c r="B2263">
+        <v>74093679</v>
+      </c>
+      <c r="C2263" t="s">
+        <v>4508</v>
+      </c>
+      <c r="D2263">
+        <v>1</v>
+      </c>
+      <c r="E2263" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2264" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2264">
+        <v>6975165332447</v>
+      </c>
+      <c r="B2264">
+        <v>74093680</v>
+      </c>
+      <c r="C2264" t="s">
+        <v>4509</v>
+      </c>
+      <c r="D2264">
+        <v>1</v>
+      </c>
+      <c r="E2264" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2265" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2265">
+        <v>6921734916785</v>
+      </c>
+      <c r="B2265">
+        <v>74093663</v>
+      </c>
+      <c r="C2265" t="s">
+        <v>4510</v>
+      </c>
+      <c r="D2265">
+        <v>1</v>
+      </c>
+      <c r="E2265" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2266" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2266">
+        <v>6935205362643</v>
+      </c>
+      <c r="B2266">
+        <v>74093664</v>
+      </c>
+      <c r="C2266" t="s">
+        <v>4511</v>
+      </c>
+      <c r="D2266">
+        <v>1</v>
+      </c>
+      <c r="E2266" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2267" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2267">
+        <v>6921734940919</v>
+      </c>
+      <c r="B2267">
+        <v>74093665</v>
+      </c>
+      <c r="C2267" t="s">
+        <v>4512</v>
+      </c>
+      <c r="D2267">
+        <v>1</v>
+      </c>
+      <c r="E2267" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2268" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2268">
+        <v>6973504009609</v>
+      </c>
+      <c r="B2268">
+        <v>74093666</v>
+      </c>
+      <c r="C2268" t="s">
+        <v>4513</v>
+      </c>
+      <c r="D2268">
+        <v>1</v>
+      </c>
+      <c r="E2268" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2269" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2269">
+        <v>6921734962782</v>
+      </c>
+      <c r="B2269">
+        <v>74093681</v>
+      </c>
+      <c r="C2269" t="s">
+        <v>4514</v>
+      </c>
+      <c r="D2269">
+        <v>1</v>
+      </c>
+      <c r="E2269" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2270" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2270">
+        <v>8991389136393</v>
+      </c>
+      <c r="B2270">
+        <v>52067727</v>
+      </c>
+      <c r="C2270" t="s">
+        <v>4515</v>
+      </c>
+      <c r="D2270">
+        <v>5</v>
+      </c>
+      <c r="E2270" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2271" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2271">
+        <v>6921734981370</v>
+      </c>
+      <c r="B2271">
+        <v>74093682</v>
+      </c>
+      <c r="C2271" t="s">
+        <v>4516</v>
+      </c>
+      <c r="D2271">
+        <v>1</v>
+      </c>
+      <c r="E2271" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2272" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2272">
+        <v>6974776203801</v>
+      </c>
+      <c r="B2272">
+        <v>74093667</v>
+      </c>
+      <c r="C2272" t="s">
+        <v>4517</v>
+      </c>
+      <c r="D2272">
+        <v>1</v>
+      </c>
+      <c r="E2272" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2273" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2273">
+        <v>6921734908902</v>
+      </c>
+      <c r="B2273">
+        <v>74093668</v>
+      </c>
+      <c r="C2273" t="s">
+        <v>4518</v>
+      </c>
+      <c r="D2273">
+        <v>1</v>
+      </c>
+      <c r="E2273" t="s">
+        <v>4504</v>
+      </c>
+    </row>
+    <row r="2274" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2274">
+        <v>3700741410676</v>
+      </c>
+      <c r="B2274">
+        <v>71093683</v>
+      </c>
+      <c r="C2274" t="s">
+        <v>4519</v>
+      </c>
+      <c r="D2274">
+        <v>1</v>
+      </c>
+      <c r="E2274" t="s">
+        <v>4520</v>
+      </c>
+    </row>
+    <row r="2275" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2275">
+        <v>3700741411062</v>
+      </c>
+      <c r="B2275">
+        <v>71093684</v>
+      </c>
+      <c r="C2275" t="s">
+        <v>4521</v>
+      </c>
+      <c r="D2275">
+        <v>1</v>
+      </c>
+      <c r="E2275" t="s">
+        <v>4520</v>
+      </c>
+    </row>
+    <row r="2276" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2276">
+        <v>3700741411246</v>
+      </c>
+      <c r="B2276">
+        <v>71093685</v>
+      </c>
+      <c r="C2276" t="s">
+        <v>4522</v>
+      </c>
+      <c r="D2276">
+        <v>1</v>
+      </c>
+      <c r="E2276" t="s">
+        <v>4520</v>
+      </c>
+    </row>
+    <row r="2277" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2277">
+        <v>3700741411741</v>
+      </c>
+      <c r="B2277">
+        <v>71093686</v>
+      </c>
+      <c r="C2277" t="s">
+        <v>4523</v>
+      </c>
+      <c r="D2277">
+        <v>1</v>
+      </c>
+      <c r="E2277" t="s">
+        <v>4520</v>
+      </c>
+    </row>
+    <row r="2278" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2278">
+        <v>3760315151701</v>
+      </c>
+      <c r="B2278">
+        <v>75093669</v>
+      </c>
+      <c r="C2278" t="s">
+        <v>4524</v>
+      </c>
+      <c r="D2278">
+        <v>24</v>
+      </c>
+      <c r="E2278" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="2279" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2279">
+        <v>6161105490920</v>
+      </c>
+      <c r="B2279">
+        <v>71093687</v>
+      </c>
+      <c r="C2279" t="s">
+        <v>4525</v>
+      </c>
+      <c r="D2279">
+        <v>56</v>
+      </c>
+      <c r="E2279" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2280" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2280">
+        <v>6161105490913</v>
+      </c>
+      <c r="B2280">
+        <v>71093688</v>
+      </c>
+      <c r="C2280" t="s">
+        <v>4526</v>
+      </c>
+      <c r="D2280">
+        <v>80</v>
+      </c>
+      <c r="E2280" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2281" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2281">
+        <v>6161105490975</v>
+      </c>
+      <c r="B2281">
+        <v>71093689</v>
+      </c>
+      <c r="C2281" t="s">
+        <v>4527</v>
+      </c>
+      <c r="D2281">
+        <v>98</v>
+      </c>
+      <c r="E2281" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2282" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2282">
+        <v>6161105490371</v>
+      </c>
+      <c r="B2282">
+        <v>71093690</v>
+      </c>
+      <c r="C2282" t="s">
+        <v>4528</v>
+      </c>
+      <c r="D2282">
+        <v>40</v>
+      </c>
+      <c r="E2282" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2283" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2283">
+        <v>6091314370907</v>
+      </c>
+      <c r="B2283">
+        <v>75093670</v>
+      </c>
+      <c r="C2283" t="s">
+        <v>4529</v>
+      </c>
+      <c r="D2283">
+        <v>25</v>
+      </c>
+      <c r="E2283" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="2284" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2284">
+        <v>3700005091825</v>
+      </c>
+      <c r="B2284">
+        <v>75093691</v>
+      </c>
+      <c r="C2284" t="s">
+        <v>4530</v>
+      </c>
+      <c r="D2284">
+        <v>35</v>
+      </c>
+      <c r="E2284" t="s">
+        <v>4531</v>
+      </c>
+    </row>
+    <row r="2285" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2285">
+        <v>3700005091894</v>
+      </c>
+      <c r="B2285">
+        <v>75093692</v>
+      </c>
+      <c r="C2285" t="s">
+        <v>4532</v>
+      </c>
+      <c r="D2285">
+        <v>35</v>
+      </c>
+      <c r="E2285" t="s">
+        <v>4531</v>
+      </c>
+    </row>
+    <row r="2286" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2286">
+        <v>5449000152848</v>
+      </c>
+      <c r="B2286">
+        <v>72093671</v>
+      </c>
+      <c r="C2286" t="s">
+        <v>4533</v>
+      </c>
+      <c r="D2286">
+        <v>6</v>
+      </c>
+      <c r="E2286" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="2287" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2287">
+        <v>42358183</v>
+      </c>
+      <c r="B2287">
+        <v>72093672</v>
+      </c>
+      <c r="C2287" t="s">
+        <v>4534</v>
+      </c>
+      <c r="D2287">
+        <v>12</v>
+      </c>
+      <c r="E2287" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="2288" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2288">
+        <v>724133052995</v>
+      </c>
+      <c r="B2288">
+        <v>71093673</v>
+      </c>
+      <c r="C2288" t="s">
+        <v>4535</v>
+      </c>
+      <c r="D2288">
+        <v>40</v>
+      </c>
+      <c r="E2288" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="2289" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2289">
+        <v>761742933031</v>
+      </c>
+      <c r="B2289">
+        <v>71093693</v>
+      </c>
+      <c r="C2289" t="s">
+        <v>4536</v>
+      </c>
+      <c r="D2289">
+        <v>40</v>
+      </c>
+      <c r="E2289" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="2290" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2290">
+        <v>761742933055</v>
+      </c>
+      <c r="B2290">
+        <v>71093694</v>
+      </c>
+      <c r="C2290" t="s">
+        <v>4537</v>
+      </c>
+      <c r="D2290">
+        <v>40</v>
+      </c>
+      <c r="E2290" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="2291" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2291">
+        <v>761742939062</v>
+      </c>
+      <c r="B2291">
+        <v>71093695</v>
+      </c>
+      <c r="C2291" t="s">
+        <v>4538</v>
+      </c>
+      <c r="D2291">
+        <v>40</v>
+      </c>
+      <c r="E2291" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="2292" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2292">
+        <v>9501100337979</v>
+      </c>
+      <c r="B2292">
+        <v>71093696</v>
+      </c>
+      <c r="C2292" t="s">
+        <v>4539</v>
+      </c>
+      <c r="D2292">
+        <v>200</v>
+      </c>
+      <c r="E2292" t="s">
+        <v>4540</v>
+      </c>
+    </row>
+    <row r="2293" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2293">
+        <v>9501100337986</v>
+      </c>
+      <c r="B2293">
+        <v>71093697</v>
+      </c>
+      <c r="C2293" t="s">
+        <v>4541</v>
+      </c>
+      <c r="D2293">
+        <v>200</v>
+      </c>
+      <c r="E2293" t="s">
+        <v>4540</v>
+      </c>
+    </row>
+    <row r="2294" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2294">
+        <v>6009678264176</v>
+      </c>
+      <c r="B2294">
+        <v>73093698</v>
+      </c>
+      <c r="C2294" t="s">
+        <v>4542</v>
+      </c>
+      <c r="D2294">
+        <v>96</v>
+      </c>
+      <c r="E2294" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2295" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2295">
+        <v>6009678264183</v>
+      </c>
+      <c r="B2295">
+        <v>73093699</v>
+      </c>
+      <c r="C2295" t="s">
+        <v>4544</v>
+      </c>
+      <c r="D2295">
+        <v>96</v>
+      </c>
+      <c r="E2295" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2296" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2296">
+        <v>6009678264190</v>
+      </c>
+      <c r="B2296">
+        <v>73093700</v>
+      </c>
+      <c r="C2296" t="s">
+        <v>4545</v>
+      </c>
+      <c r="D2296">
+        <v>96</v>
+      </c>
+      <c r="E2296" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2297" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2297">
+        <v>6009678264206</v>
+      </c>
+      <c r="B2297">
+        <v>73093701</v>
+      </c>
+      <c r="C2297" t="s">
+        <v>4546</v>
+      </c>
+      <c r="D2297">
+        <v>96</v>
+      </c>
+      <c r="E2297" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2298" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2298">
+        <v>6009678260048</v>
+      </c>
+      <c r="B2298">
+        <v>73093702</v>
+      </c>
+      <c r="C2298" t="s">
+        <v>4547</v>
+      </c>
+      <c r="D2298">
+        <v>36</v>
+      </c>
+      <c r="E2298" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2299" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2299">
+        <v>6009678260024</v>
+      </c>
+      <c r="B2299">
+        <v>73093703</v>
+      </c>
+      <c r="C2299" t="s">
+        <v>4548</v>
+      </c>
+      <c r="D2299">
+        <v>60</v>
+      </c>
+      <c r="E2299" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2300" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2300">
+        <v>6009678260260</v>
+      </c>
+      <c r="B2300">
+        <v>73093704</v>
+      </c>
+      <c r="C2300" t="s">
+        <v>4549</v>
+      </c>
+      <c r="D2300">
+        <v>150</v>
+      </c>
+      <c r="E2300" t="s">
+        <v>4543</v>
+      </c>
+    </row>
+    <row r="2301" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2301">
+        <v>3770010163039</v>
+      </c>
+      <c r="B2301">
+        <v>71093705</v>
+      </c>
+      <c r="C2301" t="s">
+        <v>4550</v>
+      </c>
+      <c r="D2301">
+        <v>1</v>
+      </c>
+      <c r="E2301" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2302" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2302">
+        <v>3770010163145</v>
+      </c>
+      <c r="B2302">
+        <v>71093706</v>
+      </c>
+      <c r="C2302" t="s">
+        <v>4552</v>
+      </c>
+      <c r="D2302">
+        <v>1</v>
+      </c>
+      <c r="E2302" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2303" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2303">
+        <v>3770010163060</v>
+      </c>
+      <c r="B2303">
+        <v>71093707</v>
+      </c>
+      <c r="C2303" t="s">
+        <v>4553</v>
+      </c>
+      <c r="D2303">
+        <v>1</v>
+      </c>
+      <c r="E2303" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2304" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2304">
+        <v>6091311381012</v>
+      </c>
+      <c r="B2304">
+        <v>71093674</v>
+      </c>
+      <c r="C2304" t="s">
+        <v>4554</v>
+      </c>
+      <c r="D2304">
+        <v>1</v>
+      </c>
+      <c r="E2304" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2305" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2305">
+        <v>2200020545118</v>
+      </c>
+      <c r="B2305">
+        <v>71093708</v>
+      </c>
+      <c r="C2305" t="s">
+        <v>4555</v>
+      </c>
+      <c r="D2305">
+        <v>1</v>
+      </c>
+      <c r="E2305" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2306" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2306">
+        <v>2200020544944</v>
+      </c>
+      <c r="B2306">
+        <v>71093709</v>
+      </c>
+      <c r="C2306" t="s">
+        <v>4556</v>
+      </c>
+      <c r="D2306">
+        <v>1</v>
+      </c>
+      <c r="E2306" t="s">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="2307" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2307">
+        <v>22160400506</v>
+      </c>
+      <c r="B2307">
+        <v>71093675</v>
+      </c>
+      <c r="C2307" t="s">
+        <v>4557</v>
+      </c>
+      <c r="D2307">
+        <v>1</v>
+      </c>
+      <c r="E2307" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2308" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2308">
+        <v>215070400500</v>
+      </c>
+      <c r="B2308">
+        <v>71093712</v>
+      </c>
+      <c r="C2308" t="s">
+        <v>4559</v>
+      </c>
+      <c r="D2308">
+        <v>1</v>
+      </c>
+      <c r="E2308" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2309" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2309">
+        <v>314020400505</v>
+      </c>
+      <c r="B2309">
+        <v>71093713</v>
+      </c>
+      <c r="C2309" t="s">
+        <v>4560</v>
+      </c>
+      <c r="D2309">
+        <v>1</v>
+      </c>
+      <c r="E2309" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2310" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2310">
+        <v>314160400502</v>
+      </c>
+      <c r="B2310">
+        <v>71093714</v>
+      </c>
+      <c r="C2310" t="s">
+        <v>4561</v>
+      </c>
+      <c r="D2310">
+        <v>1</v>
+      </c>
+      <c r="E2310" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2311" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2311">
+        <v>718030400508</v>
+      </c>
+      <c r="B2311">
+        <v>71093715</v>
+      </c>
+      <c r="C2311" t="s">
+        <v>4562</v>
+      </c>
+      <c r="D2311">
+        <v>1</v>
+      </c>
+      <c r="E2311" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2312" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2312">
+        <v>315160400509</v>
+      </c>
+      <c r="B2312">
+        <v>71093716</v>
+      </c>
+      <c r="C2312" t="s">
+        <v>4563</v>
+      </c>
+      <c r="D2312">
+        <v>1</v>
+      </c>
+      <c r="E2312" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2313" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2313">
+        <v>161160400502</v>
+      </c>
+      <c r="B2313">
+        <v>71093717</v>
+      </c>
+      <c r="C2313" t="s">
+        <v>4564</v>
+      </c>
+      <c r="D2313">
+        <v>1</v>
+      </c>
+      <c r="E2313" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2314" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2314">
+        <v>139050202000</v>
+      </c>
+      <c r="B2314">
+        <v>71093718</v>
+      </c>
+      <c r="C2314" t="s">
+        <v>4565</v>
+      </c>
+      <c r="D2314">
+        <v>1</v>
+      </c>
+      <c r="E2314" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2315" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2315">
+        <v>139130202005</v>
+      </c>
+      <c r="B2315">
+        <v>71093719</v>
+      </c>
+      <c r="C2315" t="s">
+        <v>4566</v>
+      </c>
+      <c r="D2315">
+        <v>1</v>
+      </c>
+      <c r="E2315" t="s">
+        <v>4558</v>
+      </c>
+    </row>
+    <row r="2316" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2316">
+        <v>9501046013968</v>
+      </c>
+      <c r="B2316">
+        <v>72093710</v>
+      </c>
+      <c r="C2316" t="s">
+        <v>4567</v>
+      </c>
+      <c r="D2316">
+        <v>12</v>
+      </c>
+      <c r="E2316" t="s">
+        <v>4568</v>
+      </c>
+    </row>
+    <row r="2317" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2317">
+        <v>9501046013265</v>
+      </c>
+      <c r="B2317">
+        <v>72093711</v>
+      </c>
+      <c r="C2317" t="s">
+        <v>4569</v>
+      </c>
+      <c r="D2317">
+        <v>6</v>
+      </c>
+      <c r="E2317" t="s">
+        <v>4568</v>
+      </c>
+    </row>
+    <row r="2318" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2318" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2318">
+        <v>74093546</v>
+      </c>
+      <c r="C2318" t="s">
+        <v>4570</v>
+      </c>
+      <c r="D2318">
+        <v>10</v>
+      </c>
+      <c r="E2318" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2319" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2319" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2319">
+        <v>74093547</v>
+      </c>
+      <c r="C2319" t="s">
+        <v>4572</v>
+      </c>
+      <c r="D2319">
+        <v>10</v>
+      </c>
+      <c r="E2319" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2320" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2320" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2320">
+        <v>74093548</v>
+      </c>
+      <c r="C2320" t="s">
+        <v>4573</v>
+      </c>
+      <c r="D2320">
+        <v>10</v>
+      </c>
+      <c r="E2320" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2321" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2321" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2321">
+        <v>74093549</v>
+      </c>
+      <c r="C2321" t="s">
+        <v>4574</v>
+      </c>
+      <c r="D2321">
+        <v>5</v>
+      </c>
+      <c r="E2321" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2322" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2322" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2322">
+        <v>74093550</v>
+      </c>
+      <c r="C2322" t="s">
+        <v>4575</v>
+      </c>
+      <c r="D2322">
+        <v>6</v>
+      </c>
+      <c r="E2322" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2323" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2323" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2323">
+        <v>74093551</v>
+      </c>
+      <c r="C2323" t="s">
+        <v>4576</v>
+      </c>
+      <c r="D2323">
+        <v>5</v>
+      </c>
+      <c r="E2323" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2324" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2324" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2324">
+        <v>74093552</v>
+      </c>
+      <c r="C2324" t="s">
+        <v>4577</v>
+      </c>
+      <c r="D2324">
+        <v>10</v>
+      </c>
+      <c r="E2324" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2325" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2325" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2325">
+        <v>74093553</v>
+      </c>
+      <c r="C2325" t="s">
+        <v>4578</v>
+      </c>
+      <c r="D2325">
+        <v>5</v>
+      </c>
+      <c r="E2325" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2326" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2326" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2326">
+        <v>74093554</v>
+      </c>
+      <c r="C2326" t="s">
+        <v>4579</v>
+      </c>
+      <c r="D2326">
+        <v>50</v>
+      </c>
+      <c r="E2326" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="2327" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2327" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2327">
+        <v>74093555</v>
+      </c>
+      <c r="C2327" t="s">
+        <v>4580</v>
+      </c>
+      <c r="D2327">
+        <v>50</v>
+      </c>
+      <c r="E2327" t="s">
+        <v>4571</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 26 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8873" uniqueCount="4636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8925" uniqueCount="4664">
   <si>
     <t>Code barre</t>
   </si>
@@ -13919,6 +13919,90 @@
   </si>
   <si>
     <t>SORBET MANGUE PASSION 125ML</t>
+  </si>
+  <si>
+    <t>MAKALIOKA 1KG</t>
+  </si>
+  <si>
+    <t>RAMINOARISOA MYRIAME</t>
+  </si>
+  <si>
+    <t>TSIASISA MENA 1KG</t>
+  </si>
+  <si>
+    <t>TSARAMASO MAINA FOTSY 1KG</t>
+  </si>
+  <si>
+    <t>KATSAKA 1KG</t>
+  </si>
+  <si>
+    <t>MAKALIOKA 5KG</t>
+  </si>
+  <si>
+    <t>VARY GASY MANALALONDO 5KG</t>
+  </si>
+  <si>
+    <t>LENTILLE 1KG</t>
+  </si>
+  <si>
+    <t>KABARO MAINA 1KG</t>
+  </si>
+  <si>
+    <t>VARY GASY MANALALONDO 1KG</t>
+  </si>
+  <si>
+    <t>LENTILLE 500G</t>
+  </si>
+  <si>
+    <t>TSIASISA MENA 500G</t>
+  </si>
+  <si>
+    <t>VARY MAKALIOKA D ALAOTRA 1KG</t>
+  </si>
+  <si>
+    <t>VARY MAKALIOKA D ALAOTRA 5KG</t>
+  </si>
+  <si>
+    <t>VARY GASY MANGAMILA 1KG</t>
+  </si>
+  <si>
+    <t>VARY GASY MANGAMILA 5KG</t>
+  </si>
+  <si>
+    <t>VARY MAKALIOKA D ALAOTRA 25KG</t>
+  </si>
+  <si>
+    <t>CROQ POMME 170G</t>
+  </si>
+  <si>
+    <t>CROQUETTE FEUILLETTE 200G</t>
+  </si>
+  <si>
+    <t>CROQUETTE FEUILLETTE 150G</t>
+  </si>
+  <si>
+    <t>CHIPS PATATE DOUCE 190G</t>
+  </si>
+  <si>
+    <t>CROQUETTE CHEESE 300G DELICIEUX</t>
+  </si>
+  <si>
+    <t>FRITOS MELANGE 250G DELICIEUX</t>
+  </si>
+  <si>
+    <t>FRITOS RAISIN 250G DELICIEUX</t>
+  </si>
+  <si>
+    <t>JUGL BOISSON GINGEMBRE 1L</t>
+  </si>
+  <si>
+    <t>RIZ DE TABLE MAKALIOKA SOA 5KG</t>
+  </si>
+  <si>
+    <t>SOA DISTRIBUTION</t>
+  </si>
+  <si>
+    <t>GOUTY LE SPRITZ</t>
   </si>
 </sst>
 </file>
@@ -14295,7 +14379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2221"/>
+  <dimension ref="A1:E2247"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -52055,6 +52139,448 @@
         <v>3204</v>
       </c>
     </row>
+    <row r="2222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2222">
+        <v>9326477903011</v>
+      </c>
+      <c r="B2222">
+        <v>71093828</v>
+      </c>
+      <c r="C2222" t="s">
+        <v>4636</v>
+      </c>
+      <c r="D2222">
+        <v>1</v>
+      </c>
+      <c r="E2222" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2223">
+        <v>9326477901826</v>
+      </c>
+      <c r="B2223">
+        <v>71093829</v>
+      </c>
+      <c r="C2223" t="s">
+        <v>4638</v>
+      </c>
+      <c r="D2223">
+        <v>1</v>
+      </c>
+      <c r="E2223" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2224">
+        <v>9326477906722</v>
+      </c>
+      <c r="B2224">
+        <v>71093830</v>
+      </c>
+      <c r="C2224" t="s">
+        <v>4639</v>
+      </c>
+      <c r="D2224">
+        <v>1</v>
+      </c>
+      <c r="E2224" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2225">
+        <v>9326477906326</v>
+      </c>
+      <c r="B2225">
+        <v>71093831</v>
+      </c>
+      <c r="C2225" t="s">
+        <v>4640</v>
+      </c>
+      <c r="D2225">
+        <v>1</v>
+      </c>
+      <c r="E2225" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2226">
+        <v>9326477908757</v>
+      </c>
+      <c r="B2226">
+        <v>71093832</v>
+      </c>
+      <c r="C2226" t="s">
+        <v>4641</v>
+      </c>
+      <c r="D2226">
+        <v>1</v>
+      </c>
+      <c r="E2226" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2227">
+        <v>9326477903226</v>
+      </c>
+      <c r="B2227">
+        <v>71093833</v>
+      </c>
+      <c r="C2227" t="s">
+        <v>4642</v>
+      </c>
+      <c r="D2227">
+        <v>1</v>
+      </c>
+      <c r="E2227" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2228">
+        <v>9326477908320</v>
+      </c>
+      <c r="B2228">
+        <v>71093834</v>
+      </c>
+      <c r="C2228" t="s">
+        <v>4643</v>
+      </c>
+      <c r="D2228">
+        <v>1</v>
+      </c>
+      <c r="E2228" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2229">
+        <v>9326477907323</v>
+      </c>
+      <c r="B2229">
+        <v>71093835</v>
+      </c>
+      <c r="C2229" t="s">
+        <v>4644</v>
+      </c>
+      <c r="D2229">
+        <v>1</v>
+      </c>
+      <c r="E2229" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2230">
+        <v>9326477903004</v>
+      </c>
+      <c r="B2230">
+        <v>71093836</v>
+      </c>
+      <c r="C2230" t="s">
+        <v>4645</v>
+      </c>
+      <c r="D2230">
+        <v>1</v>
+      </c>
+      <c r="E2230" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2231">
+        <v>9326477900072</v>
+      </c>
+      <c r="B2231">
+        <v>71093837</v>
+      </c>
+      <c r="C2231" t="s">
+        <v>4646</v>
+      </c>
+      <c r="D2231">
+        <v>1</v>
+      </c>
+      <c r="E2231" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2232">
+        <v>9326477906982</v>
+      </c>
+      <c r="B2232">
+        <v>71093838</v>
+      </c>
+      <c r="C2232" t="s">
+        <v>4647</v>
+      </c>
+      <c r="D2232">
+        <v>1</v>
+      </c>
+      <c r="E2232" t="s">
+        <v>4637</v>
+      </c>
+    </row>
+    <row r="2233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2233">
+        <v>3665902204627</v>
+      </c>
+      <c r="B2233">
+        <v>71093839</v>
+      </c>
+      <c r="C2233" t="s">
+        <v>4648</v>
+      </c>
+      <c r="D2233">
+        <v>1</v>
+      </c>
+      <c r="E2233" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2234">
+        <v>3665902204634</v>
+      </c>
+      <c r="B2234">
+        <v>71093840</v>
+      </c>
+      <c r="C2234" t="s">
+        <v>4649</v>
+      </c>
+      <c r="D2234">
+        <v>1</v>
+      </c>
+      <c r="E2234" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2235">
+        <v>3665902204603</v>
+      </c>
+      <c r="B2235">
+        <v>71093841</v>
+      </c>
+      <c r="C2235" t="s">
+        <v>4650</v>
+      </c>
+      <c r="D2235">
+        <v>1</v>
+      </c>
+      <c r="E2235" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2236">
+        <v>3665902204610</v>
+      </c>
+      <c r="B2236">
+        <v>71093842</v>
+      </c>
+      <c r="C2236" t="s">
+        <v>4651</v>
+      </c>
+      <c r="D2236">
+        <v>1</v>
+      </c>
+      <c r="E2236" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2237" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2237">
+        <v>3665902237625</v>
+      </c>
+      <c r="B2237">
+        <v>71093843</v>
+      </c>
+      <c r="C2237" t="s">
+        <v>4652</v>
+      </c>
+      <c r="D2237">
+        <v>1</v>
+      </c>
+      <c r="E2237" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2238" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2238">
+        <v>3665902204733</v>
+      </c>
+      <c r="B2238">
+        <v>71093844</v>
+      </c>
+      <c r="C2238" t="s">
+        <v>4653</v>
+      </c>
+      <c r="D2238">
+        <v>1</v>
+      </c>
+      <c r="E2238" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2239">
+        <v>3665902212967</v>
+      </c>
+      <c r="B2239">
+        <v>71093845</v>
+      </c>
+      <c r="C2239" t="s">
+        <v>4654</v>
+      </c>
+      <c r="D2239">
+        <v>1</v>
+      </c>
+      <c r="E2239" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2240">
+        <v>3665902239865</v>
+      </c>
+      <c r="B2240">
+        <v>71093846</v>
+      </c>
+      <c r="C2240" t="s">
+        <v>4655</v>
+      </c>
+      <c r="D2240">
+        <v>1</v>
+      </c>
+      <c r="E2240" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2241">
+        <v>3665902239872</v>
+      </c>
+      <c r="B2241">
+        <v>71093847</v>
+      </c>
+      <c r="C2241" t="s">
+        <v>4656</v>
+      </c>
+      <c r="D2241">
+        <v>1</v>
+      </c>
+      <c r="E2241" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="2242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2242">
+        <v>3770010163251</v>
+      </c>
+      <c r="B2242">
+        <v>71093848</v>
+      </c>
+      <c r="C2242" t="s">
+        <v>4657</v>
+      </c>
+      <c r="D2242">
+        <v>1</v>
+      </c>
+      <c r="E2242" t="s">
+        <v>2748</v>
+      </c>
+    </row>
+    <row r="2243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2243">
+        <v>3770010163244</v>
+      </c>
+      <c r="B2243">
+        <v>71093849</v>
+      </c>
+      <c r="C2243" t="s">
+        <v>4658</v>
+      </c>
+      <c r="D2243">
+        <v>1</v>
+      </c>
+      <c r="E2243" t="s">
+        <v>2748</v>
+      </c>
+    </row>
+    <row r="2244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2244">
+        <v>3770010163268</v>
+      </c>
+      <c r="B2244">
+        <v>71093850</v>
+      </c>
+      <c r="C2244" t="s">
+        <v>4659</v>
+      </c>
+      <c r="D2244">
+        <v>1</v>
+      </c>
+      <c r="E2244" t="s">
+        <v>2748</v>
+      </c>
+    </row>
+    <row r="2245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2245">
+        <v>9506000164632</v>
+      </c>
+      <c r="B2245">
+        <v>72093821</v>
+      </c>
+      <c r="C2245" t="s">
+        <v>4660</v>
+      </c>
+      <c r="D2245">
+        <v>6</v>
+      </c>
+      <c r="E2245" t="s">
+        <v>2338</v>
+      </c>
+    </row>
+    <row r="2246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2246">
+        <v>8961367052021</v>
+      </c>
+      <c r="B2246">
+        <v>71093822</v>
+      </c>
+      <c r="C2246" t="s">
+        <v>4661</v>
+      </c>
+      <c r="D2246">
+        <v>1</v>
+      </c>
+      <c r="E2246" t="s">
+        <v>4662</v>
+      </c>
+    </row>
+    <row r="2247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2247">
+        <v>3700005000155</v>
+      </c>
+      <c r="B2247">
+        <v>71093823</v>
+      </c>
+      <c r="C2247" t="s">
+        <v>4663</v>
+      </c>
+      <c r="D2247">
+        <v>32</v>
+      </c>
+      <c r="E2247" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Ajout CADENCIER.xlsx – 2 nouveau(x), 0 mis à jour
</commit_message>
<xml_diff>
--- a/CADENCIER.xlsx
+++ b/CADENCIER.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8925" uniqueCount="4664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8929" uniqueCount="4668">
   <si>
     <t>Code barre</t>
   </si>
@@ -14003,6 +14003,18 @@
   </si>
   <si>
     <t>GOUTY LE SPRITZ</t>
+  </si>
+  <si>
+    <t>PACK JUS DUO CERES</t>
+  </si>
+  <si>
+    <t>PANAGORA</t>
+  </si>
+  <si>
+    <t>NIDO 1+ 900G</t>
+  </si>
+  <si>
+    <t>JB</t>
   </si>
 </sst>
 </file>
@@ -14379,7 +14391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2247"/>
+  <dimension ref="A1:E2249"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -52581,6 +52593,40 @@
         <v>104</v>
       </c>
     </row>
+    <row r="2248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2248">
+        <v>3665902239810</v>
+      </c>
+      <c r="B2248">
+        <v>72094298</v>
+      </c>
+      <c r="C2248" t="s">
+        <v>4664</v>
+      </c>
+      <c r="D2248">
+        <v>1</v>
+      </c>
+      <c r="E2248" t="s">
+        <v>4665</v>
+      </c>
+    </row>
+    <row r="2249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2249">
+        <v>6001068313303</v>
+      </c>
+      <c r="B2249">
+        <v>71094299</v>
+      </c>
+      <c r="C2249" t="s">
+        <v>4666</v>
+      </c>
+      <c r="D2249">
+        <v>6</v>
+      </c>
+      <c r="E2249" t="s">
+        <v>4667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>